<commit_message>
basic 4 scales working model but ddst age visibility logic is not perfect-working on it
</commit_message>
<xml_diff>
--- a/forms/app/stage2_assessment.xlsx
+++ b/forms/app/stage2_assessment.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="survey" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="choices" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="settings" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="survey" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="choices" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="settings" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -434,7 +434,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M158"/>
+  <dimension ref="A1:N163"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -518,6 +518,11 @@
           <t>read_only</t>
         </is>
       </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>instance::type</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -5290,6 +5295,106 @@
       <c r="K158" s="2" t="inlineStr"/>
       <c r="L158" s="2" t="inlineStr"/>
       <c r="M158" s="2" t="inlineStr"/>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>begin group</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>g_supporting_docs</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>Supporting Documents / Scale Upload</t>
+        </is>
+      </c>
+      <c r="F159" t="inlineStr">
+        <is>
+          <t>field-list</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>image</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>upload_scale_image</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>Upload completed scale / assessment sheet (image)</t>
+        </is>
+      </c>
+      <c r="D160" t="inlineStr">
+        <is>
+          <t>Upload clear photos of the completed paper scale, consent form, or supporting assessment document. Accepts JPG, JPEG, PNG. For PDF use next field.</t>
+        </is>
+      </c>
+      <c r="M160" t="inlineStr">
+        <is>
+          <t>binary</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>file</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>upload_scale_pdf</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>Upload completed scale / assessment sheet (PDF)</t>
+        </is>
+      </c>
+      <c r="D161" t="inlineStr">
+        <is>
+          <t>Upload a PDF of the completed paper scale if not already uploaded as image. Accepts PDF.</t>
+        </is>
+      </c>
+      <c r="M161" t="inlineStr">
+        <is>
+          <t>binary</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>upload_caption</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>Attachment caption / description (optional)</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>end group</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>